<commit_message>
Add Bottom Line Summary sheet to Excel
New sheet with 3 summary tables (no confidence intervals):
1. Mean RT by stage and block (BL_1, BL_2, FL_1, CO_1, CO_2 + stage averages + GI)
2. Accuracy by stage and block
3. Congruency breakdown (congruent vs incongruent per stage + congruency effects)

Color-coded: green=PITCH, orange=ODOR, gray=ALL

https://claude.ai/code/session_0161wLfZ9d5BE5V6VedT4whE
</commit_message>
<xml_diff>
--- a/Garner_Analysis_Summary_All_Subjects.xlsx
+++ b/Garner_Analysis_Summary_All_Subjects.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RT by Subject-Stage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Raw Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Garner Analysis" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RT by Congruency" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Accuracy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RT by Subject-Block" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Group Means Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bottom Line Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RT by Subject-Stage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Garner Analysis" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RT by Congruency" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Accuracy" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="RT by Subject-Block" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Group Means Summary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +44,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +55,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6DCE4"/>
+        <bgColor rgb="00D6DCE4"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -83,6 +102,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,6 +485,565 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>שורה תחתונה - ממוצע RT לפי שלב ובלוק</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>קבוצה</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Baseline_1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Baseline_2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (ממוצע)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Filtering_1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Correlation_1</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Correlation_2</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Correlation (ממוצע)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>GI (F-B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>1617.9</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>1614.4</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>1615.7</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>1956.5</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>1458</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>1926</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>1686.7</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>340.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2877.1</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2909.7</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2895.2</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>3612.5</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>3122.2</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>3232.5</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>3163.8</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>717.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>2284.5</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>2300.1</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>2293.1</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>2833.2</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>2339.1</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>2617.7</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>2468.7</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>540.1</v>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>דיוק ממוצע (%) לפי שלב ובלוק</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>קבוצה</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Baseline_1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Baseline_2</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Baseline (ממוצע)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Filtering_1</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Correlation_1</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Correlation_2</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Correlation (ממוצע)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>91.7%</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>88.5%</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>90.1%</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>97.9%</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>95.8%</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>93.8%</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>94.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>86.1%</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>90.8%</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>88.4%</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>85.2%</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>88.9%</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>84.3%</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>86.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>88.7%</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>89.7%</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>89.2%</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>91.2%</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>92.2%</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>88.7%</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>90.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>ממוצע RT לפי תואם/לא-תואם ושלב</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>קבוצה</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>BL תואם</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BL לא-תואם</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FL תואם</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>FL לא-תואם</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>CO תואם</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>CO לא-תואם</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>אפקט תואמות BL</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>אפקט תואמות FL</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>אפקט תואמות CO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>1626</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1611</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>1704.6</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>2208.3</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>1458</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>1926</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>-15</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>503.7</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>3035.1</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>2755.2</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>3253.5</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>3934.8</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>2662.5</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>3692.2</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>-279.9</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>681.3</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>1029.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>2372</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>2216.8</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>2524.6</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>3122.3</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>2095.7</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>2861</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>-155.2</v>
+      </c>
+      <c r="J22" s="10" t="n">
+        <v>597.7</v>
+      </c>
+      <c r="K22" s="10" t="n">
+        <v>765.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -466,7 +1062,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -878,7 +1473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -54008,7 +54603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -54034,7 +54629,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -54553,7 +55147,6 @@
         <v>-40.24</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="C22" s="3" t="inlineStr">
         <is>
@@ -54613,7 +55206,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -54640,7 +55233,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -55220,7 +55812,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -55244,7 +55836,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -55758,7 +56349,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -58453,7 +59044,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -58478,7 +59069,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
@@ -58634,7 +59224,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>(SD)</t>
@@ -58656,7 +59245,6 @@
         <v>177.78</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -58664,7 +59252,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="2" t="inlineStr"/>
       <c r="B13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rebuild summary sheet with 5 clear tables, remove confusing Group Means
Replaced old messy sheets with clean 'שורה תחתונה' sheet:
1. Overall means by stage + GI
2. Means by stage x group (PITCH/ODOR) + GI
3. Means by stage x congruency + GI
4. Means by stage x congruency x group + GI
5. Accuracy by stage x group

https://claude.ai/code/session_0161wLfZ9d5BE5V6VedT4whE
</commit_message>
<xml_diff>
--- a/Garner_Analysis_Summary_All_Subjects.xlsx
+++ b/Garner_Analysis_Summary_All_Subjects.xlsx
@@ -7,14 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bottom Line Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="שורה תחתונה" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="RT by Subject-Stage" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Garner Analysis" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="RT by Congruency" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Accuracy" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="RT by Subject-Block" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Group Means Summary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +41,10 @@
     </font>
     <font>
       <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -94,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -120,6 +123,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,26 +489,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>שורה תחתונה - ממוצע RT לפי שלב ובלוק</t>
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>טבלה 1: ממוצע RT כללי לפי שלב</t>
         </is>
       </c>
     </row>
@@ -512,525 +512,504 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>קבוצה</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Baseline_1</t>
+          <t>Filtering</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Baseline_2</t>
+          <t>Correlation</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Baseline (ממוצע)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Filtering_1</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Correlation_1</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Correlation_2</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Correlation (ממוצע)</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
           <t>GI (F-B)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>PITCH</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>1617.9</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>1614.4</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>1615.7</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>1956.5</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>1458</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>1926</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>1686.7</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>340.8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>ODOR</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>2877.1</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>2909.7</v>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>2895.2</v>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>3612.5</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>3122.2</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>3232.5</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>3163.8</v>
-      </c>
-      <c r="J5" s="8" t="n">
-        <v>717.3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n">
+      <c r="A4" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="C6" s="10" t="n">
-        <v>2284.5</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>2300.1</v>
-      </c>
-      <c r="E6" s="10" t="n">
+      <c r="B4" s="10" t="n">
         <v>2293.1</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="C4" s="10" t="n">
         <v>2833.2</v>
       </c>
-      <c r="G6" s="10" t="n">
-        <v>2339.1</v>
-      </c>
-      <c r="H6" s="10" t="n">
-        <v>2617.7</v>
-      </c>
-      <c r="I6" s="10" t="n">
+      <c r="D4" s="10" t="n">
         <v>2468.7</v>
       </c>
-      <c r="J6" s="10" t="n">
+      <c r="E4" s="10" t="n">
         <v>540.1</v>
       </c>
     </row>
-    <row r="7"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>טבלה 2: ממוצע RT לפי שלב וקבוצה</t>
+        </is>
+      </c>
+    </row>
     <row r="8"/>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>דיוק ממוצע (%) לפי שלב ובלוק</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>קבוצה</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Filtering</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Correlation</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>GI (F-B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>1615.7</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1956.5</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1686.7</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>340.8</v>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>2895.2</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>3612.5</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>3163.8</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>717.3</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>טבלה 3: ממוצע RT לפי שלב ותואמות</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>תואמות</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Filtering</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Correlation</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>GI (F-B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>תואם</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>2372</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>2524.6</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>2095.7</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>152.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>לא תואם</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>2216.8</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>3122.3</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>2861</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>905.5</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>טבלה 4: ממוצע RT לפי שלב, תואמות וקבוצה</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>קבוצה</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>תואמות</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Baseline_1</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Baseline_2</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Baseline (ממוצע)</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Filtering_1</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Correlation_1</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Correlation_2</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Correlation (ממוצע)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Filtering</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Correlation</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>GI (F-B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>PITCH</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>תואם</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>91.7%</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>88.5%</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="D24" s="6" t="n">
+        <v>1626</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>1704.6</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>1458</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>78.59999999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>לא תואם</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1611</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>2208.3</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>1926</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>597.3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>תואם</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>3035.1</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>3253.5</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>2662.5</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>218.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>לא תואם</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>2755.2</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>3934.8</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>3692.2</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>1179.6</v>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>טבלה 5: דיוק (%) לפי שלב וקבוצה</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>קבוצה</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Filtering</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Correlation</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>כללי</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>90.1%</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>97.9%</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>95.8%</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>93.8%</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>94.8%</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>ODOR</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>93.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>86.1%</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>90.8%</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>88.4%</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>85.2%</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>88.9%</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>84.3%</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>86.6%</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>87.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>כולם</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>88.7%</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>89.7%</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>89.2%</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>91.2%</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>92.2%</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>88.7%</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>90.4%</t>
         </is>
       </c>
-    </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>ממוצע RT לפי תואם/לא-תואם ושלב</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>קבוצה</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>BL תואם</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BL לא-תואם</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>FL תואם</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>FL לא-תואם</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>CO תואם</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>CO לא-תואם</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>אפקט תואמות BL</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>אפקט תואמות FL</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>אפקט תואמות CO</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>PITCH</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>1626</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>1611</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>1704.6</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>2208.3</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>1458</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <v>1926</v>
-      </c>
-      <c r="I20" s="6" t="n">
-        <v>-15</v>
-      </c>
-      <c r="J20" s="6" t="n">
-        <v>503.7</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>ODOR</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="C21" s="8" t="n">
-        <v>3035.1</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>2755.2</v>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>3253.5</v>
-      </c>
-      <c r="F21" s="8" t="n">
-        <v>3934.8</v>
-      </c>
-      <c r="G21" s="8" t="n">
-        <v>2662.5</v>
-      </c>
-      <c r="H21" s="8" t="n">
-        <v>3692.2</v>
-      </c>
-      <c r="I21" s="8" t="n">
-        <v>-279.9</v>
-      </c>
-      <c r="J21" s="8" t="n">
-        <v>681.3</v>
-      </c>
-      <c r="K21" s="8" t="n">
-        <v>1029.7</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="C22" s="10" t="n">
-        <v>2372</v>
-      </c>
-      <c r="D22" s="10" t="n">
-        <v>2216.8</v>
-      </c>
-      <c r="E22" s="10" t="n">
-        <v>2524.6</v>
-      </c>
-      <c r="F22" s="10" t="n">
-        <v>3122.3</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>2095.7</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>2861</v>
-      </c>
-      <c r="I22" s="10" t="n">
-        <v>-155.2</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>597.7</v>
-      </c>
-      <c r="K22" s="10" t="n">
-        <v>765.3</v>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>90.1%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -59042,315 +59021,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>RT Group Means Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Baseline RT</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Filtering RT</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Correlation RT</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>GI (F-B)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>RG (B-C)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>PITCH</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>8</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1615.69</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1956.46</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1686.73</v>
-      </c>
-      <c r="F4" t="n">
-        <v>340.76</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-71.03</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>(SD)</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>771.17</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1025.15</v>
-      </c>
-      <c r="E5" t="n">
-        <v>831.02</v>
-      </c>
-      <c r="F5" t="n">
-        <v>310.91</v>
-      </c>
-      <c r="G5" t="n">
-        <v>96.61</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>ODOR</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2895.22</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3612.53</v>
-      </c>
-      <c r="E6" t="n">
-        <v>3163.81</v>
-      </c>
-      <c r="F6" t="n">
-        <v>717.3099999999999</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-268.59</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>(SD)</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>712.4400000000001</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1103.33</v>
-      </c>
-      <c r="E7" t="n">
-        <v>771.53</v>
-      </c>
-      <c r="F7" t="n">
-        <v>487.25</v>
-      </c>
-      <c r="G7" t="n">
-        <v>185.43</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>17</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2293.09</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2833.2</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2468.71</v>
-      </c>
-      <c r="F8" t="n">
-        <v>540.11</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-175.62</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>(SD)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>973.3099999999999</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1339.56</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1085.03</v>
-      </c>
-      <c r="F9" t="n">
-        <v>445.57</v>
-      </c>
-      <c r="G9" t="n">
-        <v>177.78</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Accuracy Group Means Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Baseline Acc</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Filtering Acc</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Correlation Acc</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>PITCH</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>8</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>90.1%</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>97.9%</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>94.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>ODOR</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>9</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>88.4%</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>85.2%</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>86.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>17</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>89.2%</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>91.2%</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>90.4%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>